<commit_message>
relplace school with uni
</commit_message>
<xml_diff>
--- a/_static/global/profiles.xlsx
+++ b/_static/global/profiles.xlsx
@@ -820,7 +820,11 @@
           <t>more than $4000</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T4" t="inlineStr">
         <is>
           <t>Not religious</t>
@@ -1018,7 +1022,11 @@
           <t>less than $1000</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T6" t="inlineStr">
         <is>
           <t>Not religious</t>
@@ -1620,7 +1628,11 @@
           <t>$1000-$1999</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T12" t="inlineStr">
         <is>
           <t>Orthodox</t>
@@ -2745,7 +2757,11 @@
           <t>less than $1000</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr">
         <is>
           <t>Protestant</t>
@@ -3355,7 +3371,11 @@
           <t>less than $1000</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr"/>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T29" t="inlineStr">
         <is>
           <t>Other</t>
@@ -5502,7 +5522,11 @@
           <t>$3000-$3999</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T50" t="inlineStr">
         <is>
           <t>Other</t>
@@ -6112,7 +6136,11 @@
           <t>$2000-$2999</t>
         </is>
       </c>
-      <c r="S56" t="inlineStr"/>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T56" t="inlineStr">
         <is>
           <t>Catholic</t>
@@ -7744,7 +7772,11 @@
           <t>less than $1000</t>
         </is>
       </c>
-      <c r="S72" t="inlineStr"/>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T72" t="inlineStr">
         <is>
           <t>Protestant</t>
@@ -13880,7 +13912,11 @@
           <t>less than $1000</t>
         </is>
       </c>
-      <c r="S132" t="inlineStr"/>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T132" t="inlineStr">
         <is>
           <t>Not religious</t>
@@ -14684,7 +14720,11 @@
           <t>more than $4000</t>
         </is>
       </c>
-      <c r="S140" t="inlineStr"/>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T140" t="inlineStr">
         <is>
           <t>Protestant</t>
@@ -15805,7 +15845,11 @@
           <t>$2000-$2999</t>
         </is>
       </c>
-      <c r="S151" t="inlineStr"/>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T151" t="inlineStr">
         <is>
           <t>Other</t>
@@ -16007,7 +16051,11 @@
           <t>$2000-$2999</t>
         </is>
       </c>
-      <c r="S153" t="inlineStr"/>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T153" t="inlineStr">
         <is>
           <t>Catholic</t>
@@ -18966,7 +19014,11 @@
           <t>$3000-$3999</t>
         </is>
       </c>
-      <c r="S182" t="inlineStr"/>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T182" t="inlineStr">
         <is>
           <t>Protestant</t>
@@ -20915,7 +20967,11 @@
           <t>$1000-$1999</t>
         </is>
       </c>
-      <c r="S201" t="inlineStr"/>
+      <c r="S201" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T201" t="inlineStr">
         <is>
           <t>Catholic</t>
@@ -21117,7 +21173,11 @@
           <t>more than $4000</t>
         </is>
       </c>
-      <c r="S203" t="inlineStr"/>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T203" t="inlineStr">
         <is>
           <t>Catholic</t>
@@ -21830,7 +21890,11 @@
           <t>$1000-$1999</t>
         </is>
       </c>
-      <c r="S210" t="inlineStr"/>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T210" t="inlineStr">
         <is>
           <t>Protestant</t>
@@ -21929,7 +21993,11 @@
           <t>$1000-$1999</t>
         </is>
       </c>
-      <c r="S211" t="inlineStr"/>
+      <c r="S211" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T211" t="inlineStr">
         <is>
           <t>Other</t>
@@ -24072,7 +24140,11 @@
           <t>$2000-$2999</t>
         </is>
       </c>
-      <c r="S232" t="inlineStr"/>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T232" t="inlineStr">
         <is>
           <t>Not religious</t>
@@ -25086,7 +25158,11 @@
           <t>$3000-$3999</t>
         </is>
       </c>
-      <c r="S242" t="inlineStr"/>
+      <c r="S242" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
       <c r="T242" t="inlineStr">
         <is>
           <t>Catholic</t>

</xml_diff>